<commit_message>
回退 'Pull Request !2 : 9.3夜'
</commit_message>
<xml_diff>
--- a/Excel/Test/Test.xlsx
+++ b/Excel/Test/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityWork\zhou-master\Excel\Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC081F18-D63C-42BB-A1CE-2CF2B38F137C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0335DFAF-2BC6-46E8-A103-940B75FE318C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24144" windowHeight="14447" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24144" windowHeight="14447" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CardData" sheetId="10" r:id="rId1"/>
@@ -323,7 +323,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="593">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="595">
   <si>
     <t>Id</t>
   </si>
@@ -1216,9 +1216,6 @@
     <t>AttackPoint</t>
   </si>
   <si>
-    <t>AttackRange</t>
-  </si>
-  <si>
     <t>AttackAreaWithMain</t>
   </si>
   <si>
@@ -1325,9 +1322,6 @@
   </si>
   <si>
     <t>Bullet</t>
-  </si>
-  <si>
-    <t>ShootPoint</t>
   </si>
   <si>
     <t>Modifys</t>
@@ -1885,10 +1879,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>Skill_2_Loop_A,Skill_2_Loop_B</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
     <t>小弟普攻</t>
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
@@ -1925,9 +1915,6 @@
   <si>
     <t>治愈</t>
     <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>塞雷娅击中</t>
   </si>
   <si>
     <t>{"DamageBase":1,"TriggerTime":0.5,"HpLess":0.5,"HpLessRate":1.5}</t>
@@ -2101,10 +2088,6 @@
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
   <si>
-    <t>{"MoveHeight":0,"MaxLinkNum":6,"ReductionRate":0.25,"SkillId":"CCB弹道索敌","CanBack":1,"ShowRange":1,"Color":"#ed3333"}</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
     <t>涨潮</t>
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
@@ -2145,10 +2128,6 @@
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
   <si>
-    <t>召唤地板</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
     <t>潮起</t>
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
@@ -2189,6 +2168,37 @@
   </si>
   <si>
     <t>自己入场</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>agoat2_skill_03_buff_01</t>
+  </si>
+  <si>
+    <t>纯烬艾雅法拉3加成</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>纯烬艾雅法拉3加成</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>enemy_1350_mgcshp_2</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>ShootPoint</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>C_Head</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>AttackRange</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>{"MoveHeight":0.5,"MaxLinkNum":-1,"SkillId":"CCB弹道索敌","CanBack":1}</t>
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
 </sst>
@@ -3274,8 +3284,8 @@
       <c r="B5" t="s">
         <v>135</v>
       </c>
-      <c r="F5" t="s">
-        <v>136</v>
+      <c r="F5" s="2" t="s">
+        <v>590</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -3323,17 +3333,15 @@
       <c r="AK5" t="s">
         <v>137</v>
       </c>
-      <c r="AL5" s="2" t="s">
-        <v>580</v>
-      </c>
-      <c r="AM5" s="2" t="s">
-        <v>581</v>
-      </c>
+      <c r="AL5" t="s">
+        <v>377</v>
+      </c>
+      <c r="AM5" s="2"/>
       <c r="AN5" s="2" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="AO5" s="2" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="AQ5" t="s">
         <v>138</v>
@@ -3391,19 +3399,23 @@
       </c>
     </row>
     <row r="6" spans="1:76" x14ac:dyDescent="0.25">
-      <c r="AM6" s="2" t="s">
-        <v>504</v>
-      </c>
+      <c r="F6" t="s">
+        <v>136</v>
+      </c>
+      <c r="AL6" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="AM6" s="2"/>
     </row>
     <row r="7" spans="1:76" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="E7" s="1">
         <v>1150</v>
@@ -3440,22 +3452,22 @@
         <v>0.75</v>
       </c>
       <c r="AJ7" s="1" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="AK7" s="1" t="s">
         <v>137</v>
       </c>
       <c r="AL7" s="1" t="s">
-        <v>566</v>
+        <v>562</v>
       </c>
       <c r="AM7" s="1" t="s">
-        <v>565</v>
+        <v>561</v>
       </c>
       <c r="AN7" s="3" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
       <c r="AP7" s="1">
         <v>1</v>
@@ -3474,10 +3486,10 @@
         <v>enemy_1150_dsjely</v>
       </c>
       <c r="BM7" s="1" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="BN7" s="1" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="BP7"/>
       <c r="BQ7" s="1" t="s">
@@ -3487,7 +3499,7 @@
         <v>147</v>
       </c>
       <c r="BS7" s="1" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="BT7" s="1" t="s">
         <v>148</v>
@@ -3498,13 +3510,13 @@
     </row>
     <row r="9" spans="1:76" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>570</v>
+        <v>565</v>
       </c>
       <c r="B9" t="s">
-        <v>571</v>
+        <v>566</v>
       </c>
       <c r="F9" t="s">
-        <v>572</v>
+        <v>567</v>
       </c>
       <c r="G9">
         <v>10</v>
@@ -3549,20 +3561,20 @@
         <v>0</v>
       </c>
       <c r="AJ9" s="2" t="s">
-        <v>575</v>
+        <v>570</v>
       </c>
       <c r="AK9" t="s">
         <v>137</v>
       </c>
       <c r="AL9" s="2" t="s">
-        <v>588</v>
+        <v>582</v>
       </c>
       <c r="AM9" t="s">
-        <v>589</v>
+        <v>583</v>
       </c>
       <c r="AO9" s="1"/>
       <c r="AQ9" t="s">
-        <v>573</v>
+        <v>568</v>
       </c>
       <c r="AR9">
         <v>0</v>
@@ -3577,10 +3589,10 @@
         <v>0.25</v>
       </c>
       <c r="BE9" t="s">
-        <v>574</v>
+        <v>569</v>
       </c>
       <c r="BO9" s="2" t="s">
-        <v>590</v>
+        <v>584</v>
       </c>
     </row>
   </sheetData>
@@ -4092,7 +4104,7 @@
         <v>277</v>
       </c>
       <c r="AB2" s="2" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="AC2" t="s">
         <v>278</v>
@@ -4151,203 +4163,203 @@
       <c r="AU2" t="s">
         <v>296</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="AV2" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="AW2" t="s">
         <v>297</v>
       </c>
-      <c r="AW2" t="s">
+      <c r="AX2" t="s">
         <v>298</v>
       </c>
-      <c r="AX2" t="s">
+      <c r="AY2" t="s">
         <v>299</v>
       </c>
-      <c r="AY2" t="s">
+      <c r="AZ2" t="s">
         <v>300</v>
       </c>
-      <c r="AZ2" t="s">
+      <c r="BA2" t="s">
         <v>301</v>
       </c>
-      <c r="BA2" t="s">
+      <c r="BB2" t="s">
         <v>302</v>
       </c>
-      <c r="BB2" t="s">
+      <c r="BC2" t="s">
         <v>303</v>
       </c>
-      <c r="BC2" t="s">
+      <c r="BD2" t="s">
         <v>304</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BE2" t="s">
         <v>305</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BF2" t="s">
         <v>306</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BG2" t="s">
         <v>307</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BH2" t="s">
         <v>308</v>
       </c>
-      <c r="BH2" t="s">
+      <c r="BI2" t="s">
         <v>309</v>
       </c>
-      <c r="BI2" t="s">
+      <c r="BJ2" t="s">
         <v>310</v>
       </c>
-      <c r="BJ2" t="s">
+      <c r="BK2" t="s">
         <v>311</v>
       </c>
-      <c r="BK2" t="s">
+      <c r="BL2" t="s">
         <v>312</v>
       </c>
-      <c r="BL2" t="s">
+      <c r="BM2" t="s">
         <v>313</v>
       </c>
-      <c r="BM2" t="s">
+      <c r="BN2" t="s">
         <v>314</v>
-      </c>
-      <c r="BN2" t="s">
-        <v>315</v>
       </c>
       <c r="BO2" t="s">
         <v>85</v>
       </c>
       <c r="BP2" t="s">
+        <v>315</v>
+      </c>
+      <c r="BQ2" t="s">
         <v>316</v>
       </c>
-      <c r="BQ2" t="s">
+      <c r="BR2" t="s">
         <v>317</v>
       </c>
-      <c r="BR2" t="s">
+      <c r="BS2" t="s">
         <v>318</v>
       </c>
-      <c r="BS2" t="s">
+      <c r="BT2" t="s">
         <v>319</v>
-      </c>
-      <c r="BT2" t="s">
-        <v>320</v>
       </c>
       <c r="BU2" t="s">
         <v>101</v>
       </c>
       <c r="BV2" t="s">
+        <v>320</v>
+      </c>
+      <c r="BW2" t="s">
         <v>321</v>
       </c>
-      <c r="BW2" t="s">
+      <c r="BX2" t="s">
         <v>322</v>
       </c>
-      <c r="BX2" t="s">
+      <c r="BY2" t="s">
         <v>323</v>
       </c>
-      <c r="BY2" t="s">
+      <c r="BZ2" t="s">
         <v>324</v>
       </c>
-      <c r="BZ2" t="s">
+      <c r="CA2" t="s">
         <v>325</v>
       </c>
-      <c r="CA2" t="s">
+      <c r="CB2" t="s">
         <v>326</v>
       </c>
-      <c r="CB2" t="s">
+      <c r="CC2" t="s">
         <v>327</v>
       </c>
-      <c r="CC2" t="s">
+      <c r="CD2" t="s">
         <v>328</v>
       </c>
-      <c r="CD2" t="s">
+      <c r="CE2" t="s">
         <v>329</v>
       </c>
-      <c r="CE2" t="s">
+      <c r="CF2" t="s">
         <v>330</v>
       </c>
-      <c r="CF2" t="s">
+      <c r="CG2" t="s">
         <v>331</v>
       </c>
-      <c r="CG2" t="s">
+      <c r="CH2" t="s">
         <v>332</v>
       </c>
-      <c r="CH2" t="s">
+      <c r="CI2" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="CJ2" t="s">
         <v>333</v>
       </c>
-      <c r="CI2" t="s">
+      <c r="CK2" t="s">
         <v>334</v>
       </c>
-      <c r="CJ2" t="s">
+      <c r="CL2" t="s">
         <v>335</v>
       </c>
-      <c r="CK2" t="s">
+      <c r="CM2" t="s">
         <v>336</v>
       </c>
-      <c r="CL2" t="s">
+      <c r="CN2" t="s">
         <v>337</v>
       </c>
-      <c r="CM2" t="s">
+      <c r="CO2" t="s">
         <v>338</v>
       </c>
-      <c r="CN2" t="s">
+      <c r="CP2" t="s">
         <v>339</v>
       </c>
-      <c r="CO2" t="s">
+      <c r="CQ2" t="s">
         <v>340</v>
       </c>
-      <c r="CP2" t="s">
+      <c r="CR2" t="s">
         <v>341</v>
       </c>
-      <c r="CQ2" t="s">
+      <c r="CS2" t="s">
         <v>342</v>
       </c>
-      <c r="CR2" t="s">
+      <c r="CT2" t="s">
         <v>343</v>
       </c>
-      <c r="CS2" t="s">
+      <c r="CU2" t="s">
         <v>344</v>
       </c>
-      <c r="CT2" t="s">
+      <c r="CV2" t="s">
         <v>345</v>
       </c>
-      <c r="CU2" t="s">
+      <c r="CW2" t="s">
         <v>346</v>
       </c>
-      <c r="CV2" t="s">
+      <c r="CX2" t="s">
         <v>347</v>
       </c>
-      <c r="CW2" t="s">
+      <c r="CY2" t="s">
         <v>348</v>
       </c>
-      <c r="CX2" t="s">
+      <c r="CZ2" t="s">
         <v>349</v>
       </c>
-      <c r="CY2" t="s">
+      <c r="DA2" t="s">
         <v>350</v>
       </c>
-      <c r="CZ2" t="s">
+      <c r="DB2" t="s">
         <v>351</v>
       </c>
-      <c r="DA2" t="s">
+      <c r="DC2" t="s">
         <v>352</v>
       </c>
-      <c r="DB2" t="s">
+      <c r="DD2" t="s">
         <v>353</v>
       </c>
-      <c r="DC2" t="s">
+      <c r="DE2" t="s">
         <v>354</v>
       </c>
-      <c r="DD2" t="s">
+      <c r="DF2" t="s">
         <v>355</v>
       </c>
-      <c r="DE2" t="s">
+      <c r="DG2" t="s">
         <v>356</v>
       </c>
-      <c r="DF2" t="s">
+      <c r="DH2" t="s">
         <v>357</v>
       </c>
-      <c r="DG2" t="s">
+      <c r="DI2" t="s">
         <v>358</v>
-      </c>
-      <c r="DH2" t="s">
-        <v>359</v>
-      </c>
-      <c r="DI2" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="3" spans="1:113" x14ac:dyDescent="0.25">
@@ -4376,13 +4388,13 @@
         <v>124</v>
       </c>
       <c r="J3" t="s">
+        <v>359</v>
+      </c>
+      <c r="K3" t="s">
+        <v>360</v>
+      </c>
+      <c r="L3" t="s">
         <v>361</v>
-      </c>
-      <c r="K3" t="s">
-        <v>362</v>
-      </c>
-      <c r="L3" t="s">
-        <v>363</v>
       </c>
       <c r="M3" t="s">
         <v>127</v>
@@ -4445,7 +4457,7 @@
         <v>124</v>
       </c>
       <c r="AG3" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="AH3" t="s">
         <v>124</v>
@@ -4469,10 +4481,10 @@
         <v>124</v>
       </c>
       <c r="AO3" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="AP3" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="AQ3" t="s">
         <v>2</v>
@@ -4484,7 +4496,7 @@
         <v>2</v>
       </c>
       <c r="AT3" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="AU3" t="s">
         <v>124</v>
@@ -4496,7 +4508,7 @@
         <v>124</v>
       </c>
       <c r="AX3" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="AY3" t="s">
         <v>124</v>
@@ -4526,7 +4538,7 @@
         <v>124</v>
       </c>
       <c r="BH3" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="BI3" t="s">
         <v>124</v>
@@ -4553,10 +4565,10 @@
         <v>128</v>
       </c>
       <c r="BQ3" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="BR3" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="BS3" t="s">
         <v>125</v>
@@ -4577,19 +4589,19 @@
         <v>127</v>
       </c>
       <c r="BY3" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="BZ3" t="s">
         <v>124</v>
       </c>
       <c r="CA3" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="CB3" t="s">
         <v>129</v>
       </c>
       <c r="CC3" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="CD3" t="s">
         <v>129</v>
@@ -4601,19 +4613,19 @@
         <v>129</v>
       </c>
       <c r="CG3" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="CH3" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="CI3" t="s">
         <v>2</v>
       </c>
       <c r="CJ3" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="CK3" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="CL3" t="s">
         <v>134</v>
@@ -4634,7 +4646,7 @@
         <v>133</v>
       </c>
       <c r="CR3" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="CS3" t="s">
         <v>133</v>
@@ -4646,28 +4658,28 @@
         <v>134</v>
       </c>
       <c r="CV3" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="CW3" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="CX3" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="CY3" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="CZ3" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="DA3" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="DB3" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="DC3" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="DD3" t="s">
         <v>124</v>
@@ -4690,30 +4702,30 @@
     </row>
     <row r="4" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="6" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>377</v>
+      </c>
+      <c r="C6" t="s">
+        <v>378</v>
+      </c>
+      <c r="K6" t="s">
         <v>379</v>
-      </c>
-      <c r="C6" t="s">
-        <v>380</v>
-      </c>
-      <c r="K6" t="s">
-        <v>381</v>
       </c>
       <c r="AC6">
         <v>2</v>
       </c>
       <c r="AO6" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="AV6">
         <v>8</v>
       </c>
       <c r="AX6" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="AZ6">
         <v>1</v>
@@ -4721,49 +4733,58 @@
       <c r="BD6">
         <v>1</v>
       </c>
-      <c r="CB6" s="2" t="s">
-        <v>512</v>
+      <c r="CB6" t="s">
+        <v>61</v>
       </c>
       <c r="CG6" t="s">
-        <v>384</v>
-      </c>
-      <c r="CH6" s="2" t="s">
-        <v>514</v>
-      </c>
-      <c r="CI6" t="s">
-        <v>386</v>
+        <v>382</v>
+      </c>
+      <c r="CH6" t="s">
+        <v>427</v>
+      </c>
+      <c r="CI6" s="2" t="s">
+        <v>592</v>
       </c>
       <c r="CJ6" s="2" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="CN6" s="2" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="CR6">
         <v>12</v>
       </c>
       <c r="CU6" s="2" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="CY6" t="s">
-        <v>387</v>
+        <v>385</v>
+      </c>
+      <c r="DD6">
+        <v>1</v>
+      </c>
+      <c r="DG6">
+        <v>1</v>
+      </c>
+      <c r="DH6">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
       <c r="C7" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="J7" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K7" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="R7" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
       <c r="AC7">
         <v>2</v>
@@ -4772,37 +4793,40 @@
         <v>1</v>
       </c>
       <c r="AO7" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="AV7">
-        <v>2.5</v>
+        <v>8</v>
       </c>
       <c r="BD7">
         <v>99</v>
       </c>
+      <c r="CH7" s="2" t="s">
+        <v>511</v>
+      </c>
       <c r="CU7" s="2"/>
     </row>
     <row r="8" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>388</v>
+      </c>
+      <c r="C8" t="s">
+        <v>389</v>
+      </c>
+      <c r="K8" t="s">
+        <v>387</v>
+      </c>
+      <c r="L8" t="s">
         <v>390</v>
-      </c>
-      <c r="C8" t="s">
-        <v>391</v>
-      </c>
-      <c r="K8" t="s">
-        <v>389</v>
-      </c>
-      <c r="L8" t="s">
-        <v>392</v>
       </c>
       <c r="AC8">
         <v>2</v>
       </c>
       <c r="AO8" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="AX8" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="AZ8">
         <v>0</v>
@@ -4814,30 +4838,30 @@
         <v>1</v>
       </c>
       <c r="CL8" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="CY8" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="10" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C10" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="K10" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="L10" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="AC10">
         <v>1</v>
       </c>
       <c r="AG10" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="BD10">
         <v>1</v>
@@ -4846,33 +4870,33 @@
         <v>0.1</v>
       </c>
       <c r="CN10" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="12" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="K12" s="2" t="s">
         <v>484</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>491</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>486</v>
       </c>
       <c r="AC12">
         <v>2</v>
       </c>
       <c r="AO12" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="AV12">
         <v>8</v>
       </c>
       <c r="AX12" s="2" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="AZ12">
         <v>2.5</v>
@@ -4894,51 +4918,51 @@
         <v>1</v>
       </c>
       <c r="BY12" s="2" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="CB12" t="s">
         <v>61</v>
       </c>
       <c r="CG12" t="s">
+        <v>382</v>
+      </c>
+      <c r="CH12" t="s">
+        <v>427</v>
+      </c>
+      <c r="CI12" t="s">
         <v>384</v>
       </c>
-      <c r="CH12" t="s">
-        <v>429</v>
-      </c>
-      <c r="CI12" t="s">
-        <v>386</v>
-      </c>
       <c r="CJ12" s="2" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="CN12" s="2" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
       <c r="CU12" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="CY12" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="13" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="AC13">
         <v>1</v>
       </c>
       <c r="AG13" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="BD13">
         <v>1</v>
@@ -4956,10 +4980,10 @@
         <v>1</v>
       </c>
       <c r="BY13" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="CN13" s="2" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="CO13">
         <v>200</v>
@@ -4974,22 +4998,22 @@
     </row>
     <row r="14" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="AC14">
         <v>1</v>
       </c>
       <c r="AG14" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="BD14">
         <v>1</v>
@@ -5007,43 +5031,43 @@
         <v>1</v>
       </c>
       <c r="BY14" s="2" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="CN14" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="CU14" s="2" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
     </row>
     <row r="16" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="AC16">
         <v>2</v>
       </c>
       <c r="AO16" s="2" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="AR16" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="AV16">
         <v>8</v>
       </c>
       <c r="AX16" s="2" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
       <c r="AZ16">
         <v>1.5</v>
@@ -5056,10 +5080,10 @@
       </c>
       <c r="BY16" s="2"/>
       <c r="CH16" s="2" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="CN16" s="2" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="CO16">
         <v>-50</v>
@@ -5071,25 +5095,25 @@
         <v>3</v>
       </c>
       <c r="CU16" s="2" t="s">
-        <v>568</v>
+        <v>564</v>
       </c>
     </row>
     <row r="17" spans="1:112" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="J17" s="2"/>
       <c r="K17" s="2" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>559</v>
+        <v>555</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="AC17">
         <v>2</v>
@@ -5105,34 +5129,34 @@
       </c>
       <c r="BY17" s="2"/>
       <c r="CU17" s="2" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
     </row>
     <row r="18" spans="1:112" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="AC18">
         <v>2</v>
       </c>
       <c r="AO18" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="AR18" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="AV18">
         <v>3.5</v>
       </c>
       <c r="AX18" s="2" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="AZ18">
         <v>1</v>
@@ -5145,45 +5169,45 @@
         <v>61</v>
       </c>
       <c r="CG18" t="s">
+        <v>382</v>
+      </c>
+      <c r="CH18" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="CI18" t="s">
         <v>384</v>
       </c>
-      <c r="CH18" s="2" t="s">
-        <v>514</v>
-      </c>
-      <c r="CI18" t="s">
-        <v>386</v>
-      </c>
       <c r="CN18" s="2" t="s">
-        <v>562</v>
+        <v>558</v>
       </c>
       <c r="CO18">
         <v>-0.8</v>
       </c>
       <c r="CU18" s="2" t="s">
-        <v>563</v>
+        <v>559</v>
       </c>
       <c r="CY18" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="19" spans="1:112" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="AC19">
         <v>1</v>
       </c>
       <c r="AG19" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="BD19">
         <v>1</v>
@@ -5201,10 +5225,10 @@
         <v>1</v>
       </c>
       <c r="BY19" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="CN19" s="2" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="CO19">
         <v>100</v>
@@ -5215,16 +5239,16 @@
     </row>
     <row r="20" spans="1:112" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="I20">
         <v>1</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="AC20">
         <v>1</v>
@@ -5233,10 +5257,10 @@
         <v>1</v>
       </c>
       <c r="AG20" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="AX20" s="2" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="AZ20">
         <v>0.05</v>
@@ -5251,7 +5275,7 @@
         <v>0.5</v>
       </c>
       <c r="CY20" s="2" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="DD20">
         <v>1</v>
@@ -5265,16 +5289,16 @@
     </row>
     <row r="22" spans="1:112" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>578</v>
+        <v>573</v>
       </c>
       <c r="X22">
         <v>1</v>
@@ -5295,25 +5319,25 @@
         <v>1</v>
       </c>
       <c r="BY22" s="2" t="s">
-        <v>579</v>
+        <v>574</v>
       </c>
       <c r="CU22" s="2" t="s">
-        <v>586</v>
+        <v>580</v>
       </c>
     </row>
     <row r="23" spans="1:112" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>582</v>
+        <v>576</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>583</v>
+        <v>577</v>
       </c>
       <c r="J23" s="2"/>
       <c r="K23" s="2" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>592</v>
+        <v>586</v>
       </c>
       <c r="AC23">
         <v>7</v>
@@ -5322,7 +5346,7 @@
         <v>1</v>
       </c>
       <c r="AG23" s="2" t="s">
-        <v>584</v>
+        <v>578</v>
       </c>
       <c r="AN23">
         <v>1</v>
@@ -5332,7 +5356,7 @@
       </c>
       <c r="BY23" s="2"/>
       <c r="CN23" s="2" t="s">
-        <v>585</v>
+        <v>579</v>
       </c>
       <c r="CR23">
         <v>10</v>
@@ -5424,37 +5448,37 @@
         <v>5</v>
       </c>
       <c r="E1" t="s">
+        <v>398</v>
+      </c>
+      <c r="F1" t="s">
+        <v>399</v>
+      </c>
+      <c r="G1" t="s">
         <v>400</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>401</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>402</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>403</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>404</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>405</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>406</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>407</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>408</v>
-      </c>
-      <c r="O1" t="s">
-        <v>409</v>
-      </c>
-      <c r="P1" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -5468,43 +5492,43 @@
         <v>83</v>
       </c>
       <c r="E2" t="s">
+        <v>409</v>
+      </c>
+      <c r="F2" t="s">
+        <v>410</v>
+      </c>
+      <c r="G2" t="s">
         <v>411</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>412</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>413</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>414</v>
       </c>
-      <c r="I2" t="s">
+      <c r="K2" t="s">
         <v>415</v>
-      </c>
-      <c r="J2" t="s">
-        <v>416</v>
-      </c>
-      <c r="K2" t="s">
-        <v>417</v>
       </c>
       <c r="L2" t="s">
         <v>57</v>
       </c>
       <c r="M2" t="s">
+        <v>416</v>
+      </c>
+      <c r="N2" t="s">
+        <v>417</v>
+      </c>
+      <c r="O2" t="s">
         <v>418</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P2" t="s">
         <v>419</v>
       </c>
-      <c r="O2" t="s">
-        <v>420</v>
-      </c>
-      <c r="P2" t="s">
-        <v>421</v>
-      </c>
       <c r="Q2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -5533,13 +5557,13 @@
         <v>124</v>
       </c>
       <c r="J3" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="K3" t="s">
         <v>125</v>
       </c>
       <c r="L3" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="M3" t="s">
         <v>124</v>
@@ -5548,7 +5572,7 @@
         <v>124</v>
       </c>
       <c r="O3" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="P3" t="s">
         <v>124</v>
@@ -5559,55 +5583,55 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C4" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="K4">
         <v>5</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="J5" t="s">
         <v>493</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="Q5" t="s">
         <v>494</v>
-      </c>
-      <c r="J5" t="s">
-        <v>495</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="K6">
         <v>99999</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="J7" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="K7">
         <v>12</v>
@@ -5615,80 +5639,80 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>522</v>
-      </c>
-      <c r="J8" t="s">
-        <v>523</v>
+        <v>519</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>589</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="J9" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="J10" t="s">
+        <v>534</v>
+      </c>
+      <c r="Q10" t="s">
         <v>494</v>
-      </c>
-      <c r="J10" t="s">
-        <v>538</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>560</v>
+        <v>556</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>561</v>
+        <v>557</v>
       </c>
       <c r="K11">
         <v>0.8</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
       <c r="C12" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="J12" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>550</v>
+        <v>546</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="Q14" s="2" t="s">
         <v>585</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>587</v>
-      </c>
-      <c r="Q14" s="2" t="s">
-        <v>591</v>
       </c>
     </row>
   </sheetData>
@@ -5714,7 +5738,7 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -5725,10 +5749,10 @@
         <v>51</v>
       </c>
       <c r="C2" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -5739,7 +5763,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D3" t="s">
         <v>134</v>
@@ -5747,16 +5771,16 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
       <c r="C5" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
     </row>
   </sheetData>
@@ -5768,7 +5792,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.05" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.25" customWidth="1"/>
@@ -5794,25 +5818,25 @@
         <v>53</v>
       </c>
       <c r="D2" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="E2" t="s">
         <v>76</v>
       </c>
       <c r="F2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G2" t="s">
+        <v>425</v>
+      </c>
+      <c r="H2" t="s">
         <v>426</v>
       </c>
-      <c r="G2" t="s">
-        <v>427</v>
-      </c>
-      <c r="H2" t="s">
-        <v>428</v>
-      </c>
       <c r="I2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -5841,7 +5865,7 @@
         <v>127</v>
       </c>
       <c r="I3" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="J3" t="s">
         <v>134</v>
@@ -5849,56 +5873,58 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B4" t="s">
+        <v>428</v>
+      </c>
+      <c r="C4" t="s">
         <v>529</v>
       </c>
-      <c r="B4" t="s">
-        <v>430</v>
-      </c>
-      <c r="C4" t="s">
-        <v>532</v>
-      </c>
       <c r="E4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H4">
         <v>1</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>569</v>
+        <v>594</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B5" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E5">
         <v>10</v>
       </c>
       <c r="J5" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>531</v>
-      </c>
-      <c r="C6" t="s">
-        <v>533</v>
+        <v>527</v>
       </c>
       <c r="E6">
         <v>10</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>535</v>
+        <v>531</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>528</v>
       </c>
     </row>
   </sheetData>
@@ -5910,7 +5936,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.05" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.25" customWidth="1"/>
@@ -5926,34 +5952,34 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>432</v>
+      </c>
+      <c r="C1" t="s">
+        <v>433</v>
+      </c>
+      <c r="D1" t="s">
         <v>434</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>435</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>436</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>437</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>438</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>439</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>440</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>441</v>
-      </c>
-      <c r="K1" t="s">
-        <v>442</v>
-      </c>
-      <c r="L1" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -5961,34 +5987,34 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C2" t="s">
+        <v>443</v>
+      </c>
+      <c r="D2" t="s">
         <v>444</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>445</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>446</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>447</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>448</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>449</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>450</v>
       </c>
-      <c r="I2" t="s">
-        <v>451</v>
-      </c>
-      <c r="J2" t="s">
-        <v>452</v>
-      </c>
       <c r="K2" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="L2" t="s">
         <v>103</v>
@@ -6030,6 +6056,23 @@
       </c>
       <c r="L3" t="s">
         <v>125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B4" s="2"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="B5" t="s">
+        <v>587</v>
+      </c>
+      <c r="K5">
+        <v>60</v>
+      </c>
+      <c r="L5">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -6066,22 +6109,22 @@
         <v>83</v>
       </c>
       <c r="D2" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="E2" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="F2" t="s">
         <v>85</v>
       </c>
       <c r="G2" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="H2" t="s">
         <v>284</v>
       </c>
       <c r="I2" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="J2" t="s">
         <v>58</v>
@@ -6110,7 +6153,7 @@
         <v>127</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>127</v>
@@ -6146,28 +6189,28 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>456</v>
+      </c>
+      <c r="C1" t="s">
+        <v>457</v>
+      </c>
+      <c r="D1" t="s">
         <v>458</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>459</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>460</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>461</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>462</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>463</v>
-      </c>
-      <c r="H1" t="s">
-        <v>464</v>
-      </c>
-      <c r="I1" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -6175,28 +6218,28 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>464</v>
+      </c>
+      <c r="C2" t="s">
+        <v>465</v>
+      </c>
+      <c r="D2" t="s">
         <v>466</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>467</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>468</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>469</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>470</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>471</v>
-      </c>
-      <c r="H2" t="s">
-        <v>472</v>
-      </c>
-      <c r="I2" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -6230,28 +6273,28 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" t="s">
+        <v>473</v>
+      </c>
+      <c r="E4" t="s">
+        <v>474</v>
+      </c>
+      <c r="F4" t="s">
         <v>475</v>
       </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>476</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>477</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
         <v>478</v>
-      </c>
-      <c r="H4" t="s">
-        <v>479</v>
-      </c>
-      <c r="I4" t="s">
-        <v>480</v>
       </c>
     </row>
   </sheetData>

</xml_diff>